<commit_message>
resume-mirror-eval: the mirror score is Jev's alone
Drop the code statistics from the score entirely. The mirror score is now
100 * the weighted composite of Jev's six answers and nothing else; the text
statistics survive only as the Evidence bullets and raw Details columns, with
no second roll-up number. Docs rewritten to say one Jev request per resume,
score from those answers, evidence from plain code, notes from the agent.

Mock set with Jev alone: generated mean 73, human 12; same six flagged.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJkpC3VbV552KKcrdg97YS
</commit_message>
<xml_diff>
--- a/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$E$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Details'!$A$1:$X$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Details'!$A$1:$V$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
@@ -456,7 +456,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mirror score</t>
+          <t>Mirror score (Jev)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68.5</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
@@ -510,44 +510,13 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>linh_nguyen.md</t>
+          <t>petr_ivanov.md</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>67.7</v>
+        <v>82.3</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>- 7 JD sentences appear verbatim, e.g. "- Build and maintain CI/CD pipelines in GitHub Actions and ArgoCD, enabling safe, frequent..."
-- Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
-- 9 of 9 JD acronyms present (100%), all of them
-- 36% of JD 4-word phrases reused verbatim
-- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
-- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
-- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>petr_ivanov.md</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>- 2 JD sentences appear verbatim, e.g. "- Strong understanding of observability principles, including metrics, tracing and structu..."
 - Longest shared word run is 20 words: "flux. strong understanding of observability principles including metrics tracing and structured logging. experience with service mesh technologies such ..."
@@ -558,7 +527,7 @@
 - Claims nearly every requirement, including niche ones, without matching detail</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>- The 'Mission' section is the posting's 'About the role' paragraph rewritten in the first person, including 'raise the reliability bar across the company'
 - 'Summary of Qualifications' runs through every requirement bullet in posting order as a single paragraph
@@ -566,6 +535,37 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>linh_nguyen.md</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>- 7 JD sentences appear verbatim, e.g. "- Build and maintain CI/CD pipelines in GitHub Actions and ArgoCD, enabling safe, frequent..."
+- Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
+- 9 of 9 JD acronyms present (100%), all of them
+- 36% of JD 4-word phrases reused verbatim
+- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
+- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
+- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.7</v>
+        <v>34.2</v>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15.6</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.5</v>
+        <v>14.9</v>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.3</v>
+        <v>12</v>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>8.6</v>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8.199999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6.8</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.4</v>
+        <v>1.9</v>
       </c>
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
@@ -754,33 +754,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="7" customWidth="1" min="21" max="21"/>
-    <col width="70" customWidth="1" min="22" max="22"/>
-    <col width="70" customWidth="1" min="23" max="23"/>
-    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="70" customWidth="1" min="20" max="20"/>
+    <col width="70" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -796,7 +794,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mirror score</t>
+          <t>Mirror score (Jev)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -811,95 +809,85 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Lexical</t>
+          <t>Phrase overlap</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Semantic</t>
+          <t>Longest span (words)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Phrase overlap</t>
+          <t>Order echo</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Longest span (words)</t>
+          <t>TF-IDF cos</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Order echo</t>
+          <t>Keyword cov</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>TF-IDF cos</t>
+          <t>Phrasing mirror (0-3)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Keyword cov</t>
+          <t>Requirement echo (0-3)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Phrasing mirror (0-3)</t>
+          <t>Specifics (0-3)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Requirement echo (0-3)</t>
+          <t>Generic P</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Specifics (0-3)</t>
+          <t>Posting leak P</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Generic P</t>
+          <t>Career consistent P</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Posting leak P</t>
+          <t>Verbatim JD sentences</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Career consistent P</t>
+          <t>Acronym cov</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Verbatim JD sentences</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Acronym cov</t>
+          <t>Evidence (code)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Words</t>
+          <t>LLM notes</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence (code)</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>LLM notes</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Error</t>
         </is>
@@ -917,61 +905,59 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68.5</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>1.472</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>1.594</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F2" t="n">
-        <v>47.9</v>
+        <v>0.2643</v>
       </c>
       <c r="G2" t="n">
-        <v>89.09999999999999</v>
+        <v>19</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2643</v>
+        <v>0.3404</v>
       </c>
       <c r="I2" t="n">
-        <v>19</v>
+        <v>0.4053</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3404</v>
+        <v>0.4954</v>
       </c>
       <c r="K2" t="n">
-        <v>0.4053</v>
+        <v>2.99</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4954</v>
+        <v>2.28</v>
       </c>
       <c r="M2" t="n">
-        <v>2.99</v>
+        <v>0.68</v>
       </c>
       <c r="N2" t="n">
-        <v>2.46</v>
+        <v>0.79</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7</v>
+        <v>0.99</v>
       </c>
       <c r="P2" t="n">
-        <v>0.77</v>
+        <v>0.86</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>0.84</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U2" t="n">
         <v>310</v>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>- 1 JD sentence appears verbatim, e.g. "- Expert-level Terraform skills and a strong opinion on how to structure infrastructure as..."
 - Longest shared word run is 19 words: "on eks. expert-level terraform skills and a strong opinion on how to structure infrastructure as code for multiple ..."
@@ -981,14 +967,14 @@
 - Few concrete specifics: employers, dates, numbers or named systems are thin</t>
         </is>
       </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>- 'Key Qualifications' is the posting's 'What we are looking for' list copied bullet for bullet, and the 'Nice to Have' section is the posting's own heading
 - Current role paragraph opens 'You will design, build and operate', which is addressed to an applicant, not written by one
 - Employers are 'Fintech Startup' and 'Technology Company'; no names, locations or outcomes</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -998,149 +984,59 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>linh_nguyen.md</t>
+          <t>petr_ivanov.md</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>67.7</v>
+        <v>82.3</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44</v>
+        <v>1.391</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>56.7</v>
+        <v>0.3042</v>
       </c>
       <c r="G3" t="n">
-        <v>78.7</v>
+        <v>20</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3591</v>
+        <v>0.4172</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>0.4624</v>
       </c>
       <c r="J3" t="n">
-        <v>0.58</v>
+        <v>0.5734</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4738</v>
+        <v>2.99</v>
       </c>
       <c r="L3" t="n">
-        <v>0.555</v>
+        <v>2.55</v>
       </c>
       <c r="M3" t="n">
-        <v>2.99</v>
+        <v>0.85</v>
       </c>
       <c r="N3" t="n">
-        <v>2.49</v>
+        <v>0.71</v>
       </c>
       <c r="O3" t="n">
-        <v>0.96</v>
+        <v>0.57</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.27</v>
+        <v>2</v>
       </c>
       <c r="R3" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>7</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>317</v>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>- 7 JD sentences appear verbatim, e.g. "- Build and maintain CI/CD pipelines in GitHub Actions and ArgoCD, enabling safe, frequent..."
-- Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
-- 9 of 9 JD acronyms present (100%), all of them
-- 36% of JD 4-word phrases reused verbatim
-- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="inlineStr">
-        <is>
-          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
-- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
-- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>petr_ivanov.md</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>82.90000000000001</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.3042</v>
-      </c>
-      <c r="I4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.4172</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.4624</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.5734</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="S4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U4" t="n">
         <v>311</v>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>- 2 JD sentences appear verbatim, e.g. "- Strong understanding of observability principles, including metrics, tracing and structu..."
 - Longest shared word run is 20 words: "flux. strong understanding of observability principles including metrics tracing and structured logging. experience with service mesh technologies such ..."
@@ -1151,14 +1047,92 @@
 - Claims nearly every requirement, including niche ones, without matching detail</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>- The 'Mission' section is the posting's 'About the role' paragraph rewritten in the first person, including 'raise the reliability bar across the company'
 - 'Summary of Qualifications' runs through every requirement bullet in posting order as a single paragraph
 - Two prior roles are one line each with unnamed employers</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>linh_nguyen.md</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.311</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>0.3591</v>
+      </c>
+      <c r="G4" t="n">
+        <v>80</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.4738</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>317</v>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>- 7 JD sentences appear verbatim, e.g. "- Build and maintain CI/CD pipelines in GitHub Actions and ArgoCD, enabling safe, frequent..."
+- Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
+- 9 of 9 JD acronyms present (100%), all of them
+- 36% of JD 4-word phrases reused verbatim
+- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
+- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
+- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1172,75 +1146,69 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8080000000000001</v>
+        <v>1.007</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>33.8</v>
+        <v>0.0549</v>
       </c>
       <c r="G5" t="n">
-        <v>69.3</v>
+        <v>8</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0549</v>
+        <v>0.539</v>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>0.2404</v>
       </c>
       <c r="J5" t="n">
-        <v>0.539</v>
+        <v>0.4541</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2404</v>
+        <v>2.82</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4541</v>
+        <v>2.54</v>
       </c>
       <c r="M5" t="n">
-        <v>2.8</v>
+        <v>0.99</v>
       </c>
       <c r="N5" t="n">
-        <v>2.55</v>
+        <v>0.48</v>
       </c>
       <c r="O5" t="n">
-        <v>0.98</v>
+        <v>0.05</v>
       </c>
       <c r="P5" t="n">
-        <v>0.48</v>
+        <v>0.92</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.92</v>
+        <v>0.778</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.778</v>
-      </c>
-      <c r="U5" t="n">
         <v>308</v>
       </c>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>- Longest shared word run is 8 words: "soc 2 type ii and pci dss compliance"
 - Few concrete specifics: employers, dates, numbers or named systems are thin
 - Claims nearly every requirement, including niche ones, without matching detail</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>- Each posting bullet is restated with a synonym swap ('Design, build and operate' becomes 'Architected and operated') but the same nine-bullet structure and order
 - Employers are 'Confidential Financial Services Company', 'Enterprise Software Organization' and 'Technology Consultancy'; no numbers anywhere
 - Phone screen: ask which company and what the transaction volume was</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1254,75 +1222,69 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
       <c r="D6" t="n">
-        <v>0.624</v>
+        <v>0.349</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>45.1</v>
+        <v>0.1521</v>
       </c>
       <c r="G6" t="n">
-        <v>48.4</v>
+        <v>12</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1521</v>
+        <v>0.6037</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>0.2672</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6037</v>
+        <v>0.4495</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2672</v>
+        <v>2.79</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4495</v>
+        <v>2.62</v>
       </c>
       <c r="M6" t="n">
-        <v>2.85</v>
+        <v>2.99</v>
       </c>
       <c r="N6" t="n">
-        <v>2.65</v>
+        <v>0.06</v>
       </c>
       <c r="O6" t="n">
-        <v>2.99</v>
+        <v>0.04</v>
       </c>
       <c r="P6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.88</v>
+        <v>0.889</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.889</v>
-      </c>
-      <c r="U6" t="n">
         <v>387</v>
       </c>
-      <c r="V6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>- Longest shared word run is 12 words: "secrets and identity using hashicorp vault and aws iam with least-privilege access"
 - 8 of 9 JD acronyms present (89%)
 - 15% of JD 4-word phrases reused verbatim</t>
         </is>
       </c>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>- Bullets follow the posting's order and wording, then append a metric to each; the metrics are all round (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
 - Named employers and dates are present, so the specifics score is high, but no metric is tied to a system, incident or timeframe
 - Phone screen: pick two of the percentages and ask how they were measured</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1332,63 +1294,57 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.7</v>
+        <v>34.2</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.239</v>
+        <v>-0.041</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>15.6</v>
+        <v>0.005</v>
       </c>
       <c r="G7" t="n">
-        <v>33.7</v>
+        <v>4</v>
       </c>
       <c r="H7" t="n">
-        <v>0.005</v>
+        <v>0.2623</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>0.0917</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2623</v>
+        <v>0.2294</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0917</v>
+        <v>1.75</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2294</v>
+        <v>1.99</v>
       </c>
       <c r="M7" t="n">
-        <v>1.73</v>
+        <v>2.96</v>
       </c>
       <c r="N7" t="n">
-        <v>1.95</v>
+        <v>0.09</v>
       </c>
       <c r="O7" t="n">
-        <v>2.95</v>
+        <v>0.22</v>
       </c>
       <c r="P7" t="n">
-        <v>0.09</v>
+        <v>0.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0.89</v>
+        <v>0.778</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.778</v>
-      </c>
-      <c r="U7" t="n">
         <v>251</v>
       </c>
-      <c r="V7" s="3" t="inlineStr"/>
-      <c r="W7" s="3" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+      <c r="T7" s="3" t="inlineStr"/>
+      <c r="U7" s="3" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1402,73 +1358,67 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15.6</v>
+        <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.595</v>
+        <v>-0.612</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>15.8</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>15.3</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
+        <v>0.4098</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.07489999999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.2385</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="Q8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.4098</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.07489999999999999</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.2385</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N8" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="O8" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.04</v>
-      </c>
       <c r="R8" t="n">
-        <v>0.92</v>
+        <v>0.889</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.889</v>
-      </c>
-      <c r="U8" t="n">
         <v>424</v>
       </c>
-      <c r="V8" s="3" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>- 8 of 9 JD acronyms present (89%)</t>
         </is>
       </c>
-      <c r="W8" s="3" t="inlineStr">
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>- Flagged only for acronym coverage; wording is the candidate's own, with tools the posting never mentions (Karpenter, Cilium, cosign, Thanos, Loki, Patroni, Strimzi)
 - Concrete detail throughout: 14 AWS accounts, ~$2B volume, 31% cost reduction with the named levers, a 200-star Terraform provider
 - Nothing here suggests the wording came from the posting</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -1478,63 +1428,57 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.5</v>
+        <v>14.9</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.638</v>
+        <v>-0.615</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>13.7</v>
+        <v>0.0025</v>
       </c>
       <c r="G9" t="n">
-        <v>15.3</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0025</v>
+        <v>0.157</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>0.157</v>
+        <v>0.2431</v>
       </c>
       <c r="K9" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2431</v>
+        <v>2.44</v>
       </c>
       <c r="M9" t="n">
-        <v>0.48</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>2.43</v>
+        <v>0.03</v>
       </c>
       <c r="O9" t="n">
-        <v>3</v>
+        <v>0.03</v>
       </c>
       <c r="P9" t="n">
-        <v>0.03</v>
+        <v>0.93</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0.93</v>
+        <v>0.778</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.778</v>
-      </c>
-      <c r="U9" t="n">
         <v>456</v>
       </c>
-      <c r="V9" s="3" t="inlineStr"/>
-      <c r="W9" s="3" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
+      <c r="T9" s="3" t="inlineStr"/>
+      <c r="U9" s="3" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -1544,63 +1488,57 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.3</v>
+        <v>12</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.645</v>
+        <v>-0.702</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>17.1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>11.6</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
+        <v>0.6236</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0473</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="Q10" t="n">
         <v>0</v>
       </c>
-      <c r="I10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.6236</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.0473</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.133</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="O10" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.07000000000000001</v>
-      </c>
       <c r="R10" t="n">
-        <v>0.9</v>
+        <v>0.333</v>
       </c>
       <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="U10" t="n">
         <v>247</v>
       </c>
-      <c r="V10" s="3" t="inlineStr"/>
-      <c r="W10" s="3" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
+      <c r="T10" s="3" t="inlineStr"/>
+      <c r="U10" s="3" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -1610,63 +1548,57 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>8.6</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.774</v>
+        <v>-0.803</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>13.1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
+        <v>0.2827</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.0621</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.1927</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.2827</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.0621</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.1927</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="O11" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.04</v>
-      </c>
       <c r="R11" t="n">
-        <v>0.9</v>
+        <v>0.444</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.444</v>
-      </c>
-      <c r="U11" t="n">
         <v>261</v>
       </c>
-      <c r="V11" s="3" t="inlineStr"/>
-      <c r="W11" s="3" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
+      <c r="T11" s="3" t="inlineStr"/>
+      <c r="U11" s="3" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -1676,63 +1608,57 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8.199999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.884</v>
+        <v>-0.877</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>10.9</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5.6</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
+        <v>0.3321</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.1376</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="M12" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="Q12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.3321</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.0351</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.1376</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="O12" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.07000000000000001</v>
-      </c>
       <c r="R12" t="n">
-        <v>0.89</v>
+        <v>0.111</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="U12" t="n">
         <v>236</v>
       </c>
-      <c r="V12" s="3" t="inlineStr"/>
-      <c r="W12" s="3" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
+      <c r="T12" s="3" t="inlineStr"/>
+      <c r="U12" s="3" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
@@ -1742,63 +1668,57 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6.8</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.9379999999999999</v>
+        <v>-1</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>11.5</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
+        <v>0.3158</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.0872</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="L13" t="n">
         <v>0</v>
       </c>
-      <c r="I13" t="n">
-        <v>3</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.3158</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.0306</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.0872</v>
-      </c>
       <c r="M13" t="n">
-        <v>0.06</v>
+        <v>2.98</v>
       </c>
       <c r="N13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="Q13" t="n">
         <v>0</v>
       </c>
-      <c r="O13" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.05</v>
-      </c>
       <c r="R13" t="n">
-        <v>0.92</v>
+        <v>0.111</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="U13" t="n">
         <v>230</v>
       </c>
-      <c r="V13" s="3" t="inlineStr"/>
-      <c r="W13" s="3" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
+      <c r="T13" s="3" t="inlineStr"/>
+      <c r="U13" s="3" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
@@ -1808,66 +1728,60 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.4</v>
+        <v>1.9</v>
       </c>
       <c r="D14" t="n">
-        <v>-1.071</v>
+        <v>-1.003</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>4.9</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>0.022</v>
       </c>
       <c r="J14" t="n">
+        <v>0.08260000000000001</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.08260000000000001</v>
-      </c>
       <c r="M14" t="n">
-        <v>0.04</v>
+        <v>2.98</v>
       </c>
       <c r="N14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="Q14" t="n">
         <v>0</v>
       </c>
-      <c r="O14" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0.05</v>
-      </c>
       <c r="R14" t="n">
-        <v>0.9</v>
+        <v>0.111</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="U14" t="n">
         <v>203</v>
       </c>
-      <c r="V14" s="3" t="inlineStr"/>
-      <c r="W14" s="3" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+      <c r="T14" s="3" t="inlineStr"/>
+      <c r="U14" s="3" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X14"/>
+  <autoFilter ref="A1:V14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1893,7 +1807,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-19T10:25:56</t>
+          <t>2026-09-19T10:34:19</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1860,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30.8</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="7">
@@ -2011,7 +1925,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"labelled": 13, "mean_score_by_label": {"ai_tailored": 60.4, "human": 12.3}, "flag_precision": 0.83, "flag_recall": 1.0, "auc": 1.0}</t>
+          <t>{"labelled": 13, "mean_score_by_label": {"ai_tailored": 73.5, "human": 11.8}, "flag_precision": 0.83, "flag_recall": 1.0, "auc": 1.0}</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2312,7 +2226,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>RESEARCH PROOF OF CONCEPT. These scores measure how closely a resume's wording tracks a job description. They do not determine whether a person used AI and make no decision about any candidate. The 'Needs human review' column exists so that a person reads the flagged rows: this is a tool for directing human review, not a substitute for it. Any use must comply with the laws, regulations and policies that apply to you; automated tools in hiring are regulated in many jurisdictions. Consult your legal team before using this on real applicants.</t>
+          <t>RESEARCH PROOF OF CONCEPT. The mirror score is TypeSafe Jev's measure of how closely a resume's wording tracks a job description. They do not determine whether a person used AI and make no decision about any candidate. The 'Needs human review' column exists so that a person reads the flagged rows: this is a tool for directing human review, not a substitute for it. Any use must comply with the laws, regulations and policies that apply to you; automated tools in hiring are regulated in many jurisdictions. Consult your legal team before using this on real applicants.</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2257,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Mirror score: 0-100 composite. Half from code statistics, half from Jev. Higher means the file's wording tracks the posting more closely. There are no high/medium/low grades on purpose.</t>
+          <t>Mirror score (Jev): 0-100, TypeSafe Jev's answers to six fixed questions, weighted as set in questions.py. Deterministic for the same input. Higher means the file's wording tracks the posting more closely. No high/medium/low grades on purpose.</t>
         </is>
       </c>
     </row>
@@ -2357,26 +2271,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Lexical: code-computed text statistics (verbatim 4-gram overlap, longest shared span, JD-order echo, TF-IDF cosine, keyword coverage).</t>
+          <t>Evidence (code): deterministic bullets from plain text statistics (verbatim sentences, longest shared run, acronym and phrase reuse, order) that a reviewer can check against the two documents. Not scored. The raw counts are in the Details columns.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Semantic: TypeSafe Jev judgments (phrasing mirror, requirement echo, concrete specifics, generic template, posting-language leak, career consistency).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Evidence (code): deterministic bullets a reviewer can check against the two documents. Not scored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>LLM notes: optional bullets from a generative model or the host agent. Anecdotal, not scored.</t>
         </is>

</xml_diff>

<commit_message>
resume-mirror-eval: three labelled analysis columns
Rename the columns so each says who produced it: Mirror score (Jev), Text
match analysis (code), AI analysis (agent). README's How it works and column
table are organized under the same three headings, the example table shows
all three side by side, and the spreadsheet's Read me says none feeds another.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJkpC3VbV552KKcrdg97YS
</commit_message>
<xml_diff>
--- a/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
@@ -461,12 +461,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Evidence (code)</t>
+          <t>Text match analysis (code)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>LLM notes</t>
+          <t>AI analysis (agent)</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>89.09999999999999</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -555,7 +555,8 @@
 - Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
 - 9 of 9 JD acronyms present (100%), all of them
 - 36% of JD 4-word phrases reused verbatim
-- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
+- Few concrete specifics: employers, dates, numbers or named systems are thin
+- Claims nearly every requirement, including niche ones, without matching detail</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -578,13 +579,12 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>69.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
           <t>- Longest shared word run is 8 words: "soc 2 type ii and pci dss compliance"
-- Few concrete specifics: employers, dates, numbers or named systems are thin
-- Claims nearly every requirement, including niche ones, without matching detail</t>
+- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>47.3</v>
+        <v>48.3</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>34.2</v>
+        <v>33.2</v>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.9</v>
+        <v>14.6</v>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
@@ -879,12 +879,12 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Evidence (code)</t>
+          <t>Text match analysis (code)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>LLM notes</t>
+          <t>AI analysis (agent)</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -905,10 +905,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>89.09999999999999</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>1.594</v>
+        <v>1.58</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -934,10 +934,10 @@
         <v>2.99</v>
       </c>
       <c r="L2" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
       <c r="M2" t="n">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="N2" t="n">
         <v>0.79</v>
@@ -946,7 +946,7 @@
         <v>0.99</v>
       </c>
       <c r="P2" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="Q2" t="n">
         <v>1</v>
@@ -991,7 +991,7 @@
         <v>82.3</v>
       </c>
       <c r="D3" t="n">
-        <v>1.391</v>
+        <v>1.392</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
@@ -1013,19 +1013,19 @@
         <v>2.99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.55</v>
+        <v>2.58</v>
       </c>
       <c r="M3" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="N3" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="O3" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="P3" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="Q3" t="n">
         <v>2</v>
@@ -1068,10 +1068,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="D4" t="n">
-        <v>1.311</v>
+        <v>1.318</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
@@ -1093,16 +1093,16 @@
         <v>2.99</v>
       </c>
       <c r="L4" t="n">
-        <v>2.48</v>
+        <v>2.53</v>
       </c>
       <c r="M4" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="N4" t="n">
         <v>0.83</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="P4" t="n">
         <v>0.92</v>
@@ -1122,7 +1122,8 @@
 - Longest shared word run is 80 words: "infrastructure as code using terraform and terragrunt with reusable modules consumed by product teams. build and maintain ci/cd ..."
 - 9 of 9 JD acronyms present (100%), all of them
 - 36% of JD 4-word phrases reused verbatim
-- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
+- Few concrete specifics: employers, dates, numbers or named systems are thin
+- Claims nearly every requirement, including niche ones, without matching detail</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -1146,10 +1147,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>69.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="D5" t="n">
-        <v>1.007</v>
+        <v>1.011</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
@@ -1168,16 +1169,16 @@
         <v>0.4541</v>
       </c>
       <c r="K5" t="n">
-        <v>2.82</v>
+        <v>2.79</v>
       </c>
       <c r="L5" t="n">
-        <v>2.54</v>
+        <v>2.48</v>
       </c>
       <c r="M5" t="n">
-        <v>0.99</v>
+        <v>0.9</v>
       </c>
       <c r="N5" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="O5" t="n">
         <v>0.05</v>
@@ -1197,8 +1198,7 @@
       <c r="T5" s="3" t="inlineStr">
         <is>
           <t>- Longest shared word run is 8 words: "soc 2 type ii and pci dss compliance"
-- Few concrete specifics: employers, dates, numbers or named systems are thin
-- Claims nearly every requirement, including niche ones, without matching detail</t>
+- Few concrete specifics: employers, dates, numbers or named systems are thin</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -1222,10 +1222,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>47.3</v>
+        <v>48.3</v>
       </c>
       <c r="D6" t="n">
-        <v>0.349</v>
+        <v>0.379</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
@@ -1244,16 +1244,16 @@
         <v>0.4495</v>
       </c>
       <c r="K6" t="n">
-        <v>2.79</v>
+        <v>2.85</v>
       </c>
       <c r="L6" t="n">
-        <v>2.62</v>
+        <v>2.65</v>
       </c>
       <c r="M6" t="n">
         <v>2.99</v>
       </c>
       <c r="N6" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O6" t="n">
         <v>0.04</v>
@@ -1294,10 +1294,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>34.2</v>
+        <v>33.2</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.041</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
@@ -1316,19 +1316,19 @@
         <v>0.2294</v>
       </c>
       <c r="K7" t="n">
-        <v>1.75</v>
+        <v>1.63</v>
       </c>
       <c r="L7" t="n">
         <v>1.99</v>
       </c>
       <c r="M7" t="n">
-        <v>2.96</v>
+        <v>2.95</v>
       </c>
       <c r="N7" t="n">
         <v>0.09</v>
       </c>
       <c r="O7" t="n">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="P7" t="n">
         <v>0.9</v>
@@ -1361,7 +1361,7 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.612</v>
+        <v>-0.613</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
@@ -1380,10 +1380,10 @@
         <v>0.2385</v>
       </c>
       <c r="K8" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="L8" t="n">
-        <v>2.45</v>
+        <v>2.39</v>
       </c>
       <c r="M8" t="n">
         <v>3</v>
@@ -1428,10 +1428,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.9</v>
+        <v>14.6</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.615</v>
+        <v>-0.625</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
@@ -1450,10 +1450,10 @@
         <v>0.2431</v>
       </c>
       <c r="K9" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="L9" t="n">
-        <v>2.44</v>
+        <v>2.43</v>
       </c>
       <c r="M9" t="n">
         <v>3</v>
@@ -1488,10 +1488,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.702</v>
+        <v>-0.699</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
@@ -1510,13 +1510,13 @@
         <v>0.133</v>
       </c>
       <c r="K10" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="L10" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="M10" t="n">
-        <v>2.86</v>
+        <v>2.87</v>
       </c>
       <c r="N10" t="n">
         <v>0.08</v>
@@ -1525,7 +1525,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="P10" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1548,10 +1548,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.803</v>
+        <v>-0.789</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
@@ -1570,10 +1570,10 @@
         <v>0.1927</v>
       </c>
       <c r="K11" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="L11" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M11" t="n">
         <v>2.99</v>
@@ -1608,10 +1608,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.877</v>
+        <v>-0.884</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
@@ -1630,10 +1630,10 @@
         <v>0.1376</v>
       </c>
       <c r="K12" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="L12" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="M12" t="n">
         <v>2.96</v>
@@ -1645,7 +1645,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="P12" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="D13" t="n">
-        <v>-1</v>
+        <v>-0.994</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
@@ -1690,13 +1690,13 @@
         <v>0.0872</v>
       </c>
       <c r="K13" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>2.98</v>
+        <v>2.97</v>
       </c>
       <c r="N13" t="n">
         <v>0.04</v>
@@ -1728,10 +1728,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="D14" t="n">
-        <v>-1.003</v>
+        <v>-1.006</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
@@ -1750,7 +1750,7 @@
         <v>0.08260000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1765,7 +1765,7 @@
         <v>0.05</v>
       </c>
       <c r="P14" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-19T10:34:19</t>
+          <t>2026-09-19T10:48:57</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="11">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"labelled": 13, "mean_score_by_label": {"ai_tailored": 73.5, "human": 11.8}, "flag_precision": 0.83, "flag_recall": 1.0, "auc": 1.0}</t>
+          <t>{"labelled": 13, "mean_score_by_label": {"ai_tailored": 73.7, "human": 11.7}, "flag_precision": 0.83, "flag_recall": 1.0, "auc": 1.0}</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2243,42 +2243,49 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Results sheet / results.csv: the five columns a reviewer needs. Details sheet / results-detail.csv: every statistic and Jev answer behind the score.</t>
+          <t>Three separate methods, one column each: Mirror score (Jev) is TypeSafe's decision model; Text match analysis (code) is exact string counting with no AI; AI analysis (agent) is the AI agent's own reading. None feeds another.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Needs human review: YES when any signal fired (mirror score at or above the review threshold, batch outlier, a code evidence bullet, a Jev flag, or the notes' review flag). Blank otherwise. It means 'a person should look at this file', not anything about the candidate.</t>
+          <t>Results sheet / results.csv: the five columns a reviewer needs. Details sheet / results-detail.csv: every statistic and Jev answer behind the score.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Mirror score (Jev): 0-100, TypeSafe Jev's answers to six fixed questions, weighted as set in questions.py. Deterministic for the same input. Higher means the file's wording tracks the posting more closely. No high/medium/low grades on purpose.</t>
+          <t>Needs human review: YES when any signal fired (mirror score at or above the review threshold, batch outlier, a code evidence bullet, a Jev flag, or the notes' review flag). Blank otherwise. It means 'a person should look at this file', not anything about the candidate.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Batch z: how many standard deviations this file sits above or below the batch mean. Batch outlier: YES past the threshold in questions.py.</t>
+          <t>Mirror score (Jev): 0-100, TypeSafe Jev's answers to six fixed questions, weighted as set in questions.py. Deterministic for the same input. Higher means the file's wording tracks the posting more closely. No high/medium/low grades on purpose.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Evidence (code): deterministic bullets from plain text statistics (verbatim sentences, longest shared run, acronym and phrase reuse, order) that a reviewer can check against the two documents. Not scored. The raw counts are in the Details columns.</t>
+          <t>Batch z: how many standard deviations this file sits above or below the batch mean. Batch outlier: YES past the threshold in questions.py.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>LLM notes: optional bullets from a generative model or the host agent. Anecdotal, not scored.</t>
+          <t>Text match analysis (code): sentences filled in by the script from exact counts (verbatim sentences, longest shared word run, acronym and phrase reuse, order). No AI writes or reads this column. Not scored. Raw counts are in the Details columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>AI analysis (agent): the AI agent's own observations after reading the resume against the posting. Judgment, not counting. Not scored; only its final review yes/no feeds the review flag.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
resume-mirror-eval: plain-sentence AI analysis
Each bullet is one complete sentence a recruiter reads once. The prompt and
SKILL.md now say so with an example of what not to do; the example notes are
rewritten in that style and the README rows refreshed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJkpC3VbV552KKcrdg97YS
</commit_message>
<xml_diff>
--- a/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
@@ -496,9 +496,9 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>- 'Key Qualifications' is the posting's 'What we are looking for' list copied bullet for bullet, and the 'Nice to Have' section is the posting's own heading
-- Current role paragraph opens 'You will design, build and operate', which is addressed to an applicant, not written by one
-- Employers are 'Fintech Startup' and 'Technology Company'; no names, locations or outcomes</t>
+          <t>- The resume's qualifications section repeats the posting's requirements list word for word, bullet by bullet
+- The current job is described as "You will design, build and operate...", which is how a posting talks to an applicant, not how a person describes their own work
+- Employers are given only as "Fintech Startup" and "Technology Company"</t>
         </is>
       </c>
     </row>
@@ -529,9 +529,9 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>- The 'Mission' section is the posting's 'About the role' paragraph rewritten in the first person, including 'raise the reliability bar across the company'
-- 'Summary of Qualifications' runs through every requirement bullet in posting order as a single paragraph
-- Two prior roles are one line each with unnamed employers</t>
+          <t>- The opening "Mission" paragraph is the posting's description of the role, reworded into the first person
+- The qualifications summary walks through every posting requirement in the posting's order as one long paragraph
+- The two earlier jobs are a single line each, with unnamed employers</t>
         </is>
       </c>
     </row>
@@ -561,9 +561,9 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
-- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
-- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
+          <t>- The nine duties listed in the posting appear as the nine bullets of the candidate's current job, in the same order and nearly the same words
+- The employers are described only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents
+- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong</t>
         </is>
       </c>
     </row>
@@ -589,9 +589,9 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting bullet is restated with a synonym swap ('Design, build and operate' becomes 'Architected and operated') but the same nine-bullet structure and order
-- Employers are 'Confidential Financial Services Company', 'Enterprise Software Organization' and 'Technology Consultancy'; no numbers anywhere
-- Phone screen: ask which company and what the transaction volume was</t>
+          <t>- Each posting duty appears as a resume bullet with a word swapped ("Design, build and operate" becomes "Architected and operated"), keeping the same nine-bullet order
+- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy"; there are no numbers anywhere
+- Phone screen: ask which company it was and how much transaction volume it handled</t>
         </is>
       </c>
     </row>
@@ -618,8 +618,9 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>- Bullets follow the posting's order and wording, then append a metric to each; the metrics are all round (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
-- Named employers and dates are present, so the specifics score is high, but no metric is tied to a system, incident or timeframe
+          <t>- The bullets follow the posting's order and wording, with a percentage added to the end of each one
+- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
+- Employers and dates are real-looking, but no number is tied to a specific system, incident or time period
 - Phone screen: pick two of the percentages and ask how they were measured</t>
         </is>
       </c>
@@ -658,9 +659,9 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only for acronym coverage; wording is the candidate's own, with tools the posting never mentions (Karpenter, Cilium, cosign, Thanos, Loki, Patroni, Strimzi)
-- Concrete detail throughout: 14 AWS accounts, ~$2B volume, 31% cost reduction with the named levers, a 200-star Terraform provider
-- Nothing here suggests the wording came from the posting</t>
+          <t>- Flagged only because most of the posting's acronyms appear; the wording is the candidate's own and mentions tools the posting never does
+- Plenty of concrete detail: 14 AWS accounts, about $2B in payment volume, a 31% cost reduction with the specific steps that got there
+- Nothing suggests the wording came from the posting</t>
         </is>
       </c>
     </row>
@@ -969,9 +970,9 @@
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>- 'Key Qualifications' is the posting's 'What we are looking for' list copied bullet for bullet, and the 'Nice to Have' section is the posting's own heading
-- Current role paragraph opens 'You will design, build and operate', which is addressed to an applicant, not written by one
-- Employers are 'Fintech Startup' and 'Technology Company'; no names, locations or outcomes</t>
+          <t>- The resume's qualifications section repeats the posting's requirements list word for word, bullet by bullet
+- The current job is described as "You will design, build and operate...", which is how a posting talks to an applicant, not how a person describes their own work
+- Employers are given only as "Fintech Startup" and "Technology Company"</t>
         </is>
       </c>
       <c r="V2" t="inlineStr"/>
@@ -1049,9 +1050,9 @@
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>- The 'Mission' section is the posting's 'About the role' paragraph rewritten in the first person, including 'raise the reliability bar across the company'
-- 'Summary of Qualifications' runs through every requirement bullet in posting order as a single paragraph
-- Two prior roles are one line each with unnamed employers</t>
+          <t>- The opening "Mission" paragraph is the posting's description of the role, reworded into the first person
+- The qualifications summary walks through every posting requirement in the posting's order as one long paragraph
+- The two earlier jobs are a single line each, with unnamed employers</t>
         </is>
       </c>
       <c r="V3" t="inlineStr"/>
@@ -1128,9 +1129,9 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>- All nine 'What you will do' bullets from the posting appear as the current-role bullets, in the posting's order, with 'Design, build and operate' kept in the imperative
-- Employers are 'Leading Fintech Company' and 'Global Technology Solutions Firm'; no cluster counts, team sizes, incident examples or dates beyond years
-- Phone screen: ask for one specific EKS upgrade they ran and what broke</t>
+          <t>- The nine duties listed in the posting appear as the nine bullets of the candidate's current job, in the same order and nearly the same words
+- The employers are described only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents
+- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong</t>
         </is>
       </c>
       <c r="V4" t="inlineStr"/>
@@ -1203,9 +1204,9 @@
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting bullet is restated with a synonym swap ('Design, build and operate' becomes 'Architected and operated') but the same nine-bullet structure and order
-- Employers are 'Confidential Financial Services Company', 'Enterprise Software Organization' and 'Technology Consultancy'; no numbers anywhere
-- Phone screen: ask which company and what the transaction volume was</t>
+          <t>- Each posting duty appears as a resume bullet with a word swapped ("Design, build and operate" becomes "Architected and operated"), keeping the same nine-bullet order
+- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy"; there are no numbers anywhere
+- Phone screen: ask which company it was and how much transaction volume it handled</t>
         </is>
       </c>
       <c r="V5" t="inlineStr"/>
@@ -1279,8 +1280,9 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>- Bullets follow the posting's order and wording, then append a metric to each; the metrics are all round (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
-- Named employers and dates are present, so the specifics score is high, but no metric is tied to a system, incident or timeframe
+          <t>- The bullets follow the posting's order and wording, with a percentage added to the end of each one
+- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
+- Employers and dates are real-looking, but no number is tied to a specific system, incident or time period
 - Phone screen: pick two of the percentages and ask how they were measured</t>
         </is>
       </c>
@@ -1413,9 +1415,9 @@
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only for acronym coverage; wording is the candidate's own, with tools the posting never mentions (Karpenter, Cilium, cosign, Thanos, Loki, Patroni, Strimzi)
-- Concrete detail throughout: 14 AWS accounts, ~$2B volume, 31% cost reduction with the named levers, a 200-star Terraform provider
-- Nothing here suggests the wording came from the posting</t>
+          <t>- Flagged only because most of the posting's acronyms appear; the wording is the candidate's own and mentions tools the posting never does
+- Plenty of concrete detail: 14 AWS accounts, about $2B in payment volume, a 31% cost reduction with the specific steps that got there
+- Nothing suggests the wording came from the posting</t>
         </is>
       </c>
       <c r="V8" t="inlineStr"/>
@@ -1940,271 +1942,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t># Senior Platform Engineer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>**Northwind Ledger** (fictional company, used for demonstration only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Remote (US) | Full-time | Platform Engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>## About the role</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Northwind Ledger builds payment reconciliation software for mid-market finance teams. The platform team owns the infrastructure, deployment tooling and observability stack that every product team ships on. We are looking for a Senior Platform Engineer to design and operate the Kubernetes platform that runs our transaction processing services, and to raise the reliability bar across the company.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>## What you will do</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>- Design, build and operate our production Kubernetes platform on AWS EKS, including cluster lifecycle, upgrades and multi-region failover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>- Own our infrastructure as code using Terraform and Terragrunt, with reusable modules consumed by product teams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>- Build and maintain CI/CD pipelines in GitHub Actions and ArgoCD, enabling safe, frequent deployments with automated rollback.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>- Define and track SLOs for critical services and lead the observability practice using Prometheus, Grafana and OpenTelemetry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>- Implement service mesh capabilities with Istio for mTLS, traffic shaping and progressive delivery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>- Manage secrets and identity using HashiCorp Vault and AWS IAM with least-privilege access patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>- Partner with security to maintain our SOC 2 Type II and PCI DSS compliance posture through automated controls and evidence collection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>- Participate in a follow-the-sun on-call rotation and lead blameless postmortems for production incidents.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>- Mentor engineers across product teams on cloud-native best practices and platform adoption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>## What we are looking for</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>- 6+ years of experience in infrastructure, SRE or platform engineering roles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>- Deep hands-on experience operating Kubernetes in production at scale, ideally on EKS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>- Expert-level Terraform skills and a strong opinion on how to structure infrastructure as code for multiple teams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>- Proficiency in Python or Go for building internal tooling and automation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>- Experience designing CI/CD pipelines with GitOps workflows using ArgoCD or Flux.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>- Strong understanding of observability principles, including metrics, tracing and structured logging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>- Experience with service mesh technologies such as Istio or Linkerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>- Familiarity with compliance frameworks such as SOC 2 and PCI DSS in a regulated environment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>- Excellent written communication skills and a track record of documenting systems for other engineers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>## Nice to have</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>- Experience with FinOps and cloud cost optimization on AWS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>- Contributions to open source projects in the cloud-native ecosystem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>- Experience running PostgreSQL or Kafka in Kubernetes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>## Compensation and benefits</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Base salary range: $175,000 to $215,000 depending on experience, plus equity. Fully remote within the United States. Health, dental and vision coverage; 401(k) match; a home office stipend; and a learning budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Northwind Ledger is an equal opportunity employer. This posting is fictional and exists only to demonstrate a resume screening methodology.</t>
-        </is>
-      </c>
+      <c r="A1" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
resume-mirror-eval: AI analysis bullets say why the observation matters
Observation plus what it suggests to a reviewer, in one sentence. Rule added
to the prompt and SKILL.md; example notes and README rows rewritten.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJkpC3VbV552KKcrdg97YS
</commit_message>
<xml_diff>
--- a/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
@@ -496,9 +496,9 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>- The resume's qualifications section repeats the posting's requirements list word for word, bullet by bullet
-- The current job is described as "You will design, build and operate...", which is how a posting talks to an applicant, not how a person describes their own work
-- Employers are given only as "Fintech Startup" and "Technology Company"</t>
+          <t>- The qualifications section repeats the posting's requirements list word for word, so it tells you what the posting asked for, not what this person has done
+- The current job is described as "You will design, build and operate...", which is how a posting addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
+- Employers are given only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
         </is>
       </c>
     </row>
@@ -529,9 +529,9 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>- The opening "Mission" paragraph is the posting's description of the role, reworded into the first person
-- The qualifications summary walks through every posting requirement in the posting's order as one long paragraph
-- The two earlier jobs are a single line each, with unnamed employers</t>
+          <t>- The opening "Mission" paragraph is the posting's own description of the role reworded into the first person, so the candidate's stated goal is the employer's text
+- The qualifications summary walks through every posting requirement in the posting's order, which is unlikely to happen by chance when someone writes from their own history
+- The two earlier jobs are one line each with unnamed employers, so there is no track record to compare the claims against</t>
         </is>
       </c>
     </row>
@@ -561,9 +561,9 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>- The nine duties listed in the posting appear as the nine bullets of the candidate's current job, in the same order and nearly the same words
-- The employers are described only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents
-- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong</t>
+          <t>- The nine duties listed in the posting appear as the nine bullets of the current job, in the same order and nearly the same words, which is what you get when a resume is written from the posting rather than from memory of the work
+- The employers are given only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents, so there is nothing here that could be checked
+- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong; someone who did the work will have a story</t>
         </is>
       </c>
     </row>
@@ -589,9 +589,9 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting duty appears as a resume bullet with a word swapped ("Design, build and operate" becomes "Architected and operated"), keeping the same nine-bullet order
-- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy"; there are no numbers anywhere
-- Phone screen: ask which company it was and how much transaction volume it handled</t>
+          <t>- Each posting duty appears as a resume bullet with one word swapped ("Design, build and operate" becomes "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
+- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and there are no numbers anywhere, so nothing can be checked
+- Phone screen: ask which company it was and how much transaction volume it handled; a vague answer would confirm the concern</t>
         </is>
       </c>
     </row>
@@ -618,10 +618,10 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>- The bullets follow the posting's order and wording, with a percentage added to the end of each one
-- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
-- Employers and dates are real-looking, but no number is tied to a specific system, incident or time period
-- Phone screen: pick two of the percentages and ask how they were measured</t>
+          <t>- The bullets follow the posting's order and wording with a percentage added to each, so the results look measured but the underlying claims are still the posting's
+- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
+- Employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
+- Phone screen: pick two of the percentages and ask how they were measured; real ones come with a story, invented ones do not</t>
         </is>
       </c>
     </row>
@@ -659,8 +659,8 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only because most of the posting's acronyms appear; the wording is the candidate's own and mentions tools the posting never does
-- Plenty of concrete detail: 14 AWS accounts, about $2B in payment volume, a 31% cost reduction with the specific steps that got there
+          <t>- Flagged only because most of the posting's acronyms appear, which is expected for someone who has this stack; the wording is the candidate's own and names tools the posting never mentions
+- The detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
 - Nothing suggests the wording came from the posting</t>
         </is>
       </c>
@@ -970,9 +970,9 @@
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>- The resume's qualifications section repeats the posting's requirements list word for word, bullet by bullet
-- The current job is described as "You will design, build and operate...", which is how a posting talks to an applicant, not how a person describes their own work
-- Employers are given only as "Fintech Startup" and "Technology Company"</t>
+          <t>- The qualifications section repeats the posting's requirements list word for word, so it tells you what the posting asked for, not what this person has done
+- The current job is described as "You will design, build and operate...", which is how a posting addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
+- Employers are given only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
         </is>
       </c>
       <c r="V2" t="inlineStr"/>
@@ -1050,9 +1050,9 @@
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>- The opening "Mission" paragraph is the posting's description of the role, reworded into the first person
-- The qualifications summary walks through every posting requirement in the posting's order as one long paragraph
-- The two earlier jobs are a single line each, with unnamed employers</t>
+          <t>- The opening "Mission" paragraph is the posting's own description of the role reworded into the first person, so the candidate's stated goal is the employer's text
+- The qualifications summary walks through every posting requirement in the posting's order, which is unlikely to happen by chance when someone writes from their own history
+- The two earlier jobs are one line each with unnamed employers, so there is no track record to compare the claims against</t>
         </is>
       </c>
       <c r="V3" t="inlineStr"/>
@@ -1129,9 +1129,9 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>- The nine duties listed in the posting appear as the nine bullets of the candidate's current job, in the same order and nearly the same words
-- The employers are described only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents
-- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong</t>
+          <t>- The nine duties listed in the posting appear as the nine bullets of the current job, in the same order and nearly the same words, which is what you get when a resume is written from the posting rather than from memory of the work
+- The employers are given only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents, so there is nothing here that could be checked
+- Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong; someone who did the work will have a story</t>
         </is>
       </c>
       <c r="V4" t="inlineStr"/>
@@ -1204,9 +1204,9 @@
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting duty appears as a resume bullet with a word swapped ("Design, build and operate" becomes "Architected and operated"), keeping the same nine-bullet order
-- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy"; there are no numbers anywhere
-- Phone screen: ask which company it was and how much transaction volume it handled</t>
+          <t>- Each posting duty appears as a resume bullet with one word swapped ("Design, build and operate" becomes "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
+- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and there are no numbers anywhere, so nothing can be checked
+- Phone screen: ask which company it was and how much transaction volume it handled; a vague answer would confirm the concern</t>
         </is>
       </c>
       <c r="V5" t="inlineStr"/>
@@ -1280,10 +1280,10 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>- The bullets follow the posting's order and wording, with a percentage added to the end of each one
-- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%
-- Employers and dates are real-looking, but no number is tied to a specific system, incident or time period
-- Phone screen: pick two of the percentages and ask how they were measured</t>
+          <t>- The bullets follow the posting's order and wording with a percentage added to each, so the results look measured but the underlying claims are still the posting's
+- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
+- Employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
+- Phone screen: pick two of the percentages and ask how they were measured; real ones come with a story, invented ones do not</t>
         </is>
       </c>
       <c r="V6" t="inlineStr"/>
@@ -1415,8 +1415,8 @@
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only because most of the posting's acronyms appear; the wording is the candidate's own and mentions tools the posting never does
-- Plenty of concrete detail: 14 AWS accounts, about $2B in payment volume, a 31% cost reduction with the specific steps that got there
+          <t>- Flagged only because most of the posting's acronyms appear, which is expected for someone who has this stack; the wording is the candidate's own and names tools the posting never mentions
+- The detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
 - Nothing suggests the wording came from the posting</t>
         </is>
       </c>

</xml_diff>

<commit_message>
resume-mirror-eval: AI analysis names source and copy on every comparison
'The resume's X section copies the JD's Y list', never a bare mapping of one
heading to another. Rule in the prompt and SKILL.md; examples rewritten.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJkpC3VbV552KKcrdg97YS
</commit_message>
<xml_diff>
--- a/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/resume-mirror-eval/mock-data/example-output/results.xlsx
@@ -496,9 +496,10 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>- The qualifications section repeats the posting's requirements list word for word, so it tells you what the posting asked for, not what this person has done
-- The current job is described as "You will design, build and operate...", which is how a posting addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
-- Employers are given only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
+          <t>- The resume's "Key Qualifications" section copies the JD's "What we are looking for" list word for word, so it tells you what the posting asked for, not what this person has done
+- The resume's "Nice to Have" section copies the JD's "Nice to have" section, heading and all, which is a posting section, not a resume section
+- The resume describes the current job as "You will design, build and operate...", which is how the JD addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
+- The resume names its employers only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
         </is>
       </c>
     </row>
@@ -529,9 +530,9 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>- The opening "Mission" paragraph is the posting's own description of the role reworded into the first person, so the candidate's stated goal is the employer's text
-- The qualifications summary walks through every posting requirement in the posting's order, which is unlikely to happen by chance when someone writes from their own history
-- The two earlier jobs are one line each with unnamed employers, so there is no track record to compare the claims against</t>
+          <t>- The resume's opening "Mission" paragraph is the JD's "About the role" paragraph reworded into the first person, so the candidate's stated goal is the employer's text
+- The resume's "Summary of Qualifications" walks through the JD's "What we are looking for" list in the JD's order, which is unlikely to happen by chance when someone writes from their own history
+- The resume gives its two earlier jobs one line each with unnamed employers, so there is no track record to compare the claims against</t>
         </is>
       </c>
     </row>
@@ -561,8 +562,8 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>- The nine duties listed in the posting appear as the nine bullets of the current job, in the same order and nearly the same words, which is what you get when a resume is written from the posting rather than from memory of the work
-- The employers are given only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents, so there is nothing here that could be checked
+          <t>- The resume's current-job bullets copy the JD's "What you will do" list: all nine duties, in the JD's order, in nearly the JD's words, which is what you get when a resume is written from the posting rather than from memory of the work
+- The resume names its employers only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no team sizes, numbers or incidents, so there is nothing here that could be checked
 - Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong; someone who did the work will have a story</t>
         </is>
       </c>
@@ -589,8 +590,8 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting duty appears as a resume bullet with one word swapped ("Design, build and operate" becomes "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
-- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and there are no numbers anywhere, so nothing can be checked
+          <t>- The resume's current-job bullets restate the JD's "What you will do" list with one word swapped per bullet (the JD's "Design, build and operate" becomes the resume's "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
+- The resume names its employers as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and gives no numbers anywhere, so nothing can be checked
 - Phone screen: ask which company it was and how much transaction volume it handled; a vague answer would confirm the concern</t>
         </is>
       </c>
@@ -618,9 +619,9 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>- The bullets follow the posting's order and wording with a percentage added to each, so the results look measured but the underlying claims are still the posting's
-- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
-- Employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
+          <t>- The resume's current-job bullets follow the JD's "What you will do" list in order and wording, with a percentage added to the end of each, so the results look measured but the underlying claims are still the posting's
+- Every percentage in the resume is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
+- The resume's employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
 - Phone screen: pick two of the percentages and ask how they were measured; real ones come with a story, invented ones do not</t>
         </is>
       </c>
@@ -659,9 +660,9 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only because most of the posting's acronyms appear, which is expected for someone who has this stack; the wording is the candidate's own and names tools the posting never mentions
-- The detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
-- Nothing suggests the wording came from the posting</t>
+          <t>- Flagged only because most of the JD's acronyms appear in the resume, which is expected for someone who has this stack; the resume's wording is its own and names tools the JD never mentions
+- The resume's detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
+- Nothing suggests the resume's wording came from the JD</t>
         </is>
       </c>
     </row>
@@ -970,9 +971,10 @@
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>- The qualifications section repeats the posting's requirements list word for word, so it tells you what the posting asked for, not what this person has done
-- The current job is described as "You will design, build and operate...", which is how a posting addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
-- Employers are given only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
+          <t>- The resume's "Key Qualifications" section copies the JD's "What we are looking for" list word for word, so it tells you what the posting asked for, not what this person has done
+- The resume's "Nice to Have" section copies the JD's "Nice to have" section, heading and all, which is a posting section, not a resume section
+- The resume describes the current job as "You will design, build and operate...", which is how the JD addresses an applicant, not how a person describes their own work; that phrasing usually means text was pasted from the posting
+- The resume names its employers only as "Fintech Startup" and "Technology Company", so the work history cannot be verified as written</t>
         </is>
       </c>
       <c r="V2" t="inlineStr"/>
@@ -1050,9 +1052,9 @@
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>- The opening "Mission" paragraph is the posting's own description of the role reworded into the first person, so the candidate's stated goal is the employer's text
-- The qualifications summary walks through every posting requirement in the posting's order, which is unlikely to happen by chance when someone writes from their own history
-- The two earlier jobs are one line each with unnamed employers, so there is no track record to compare the claims against</t>
+          <t>- The resume's opening "Mission" paragraph is the JD's "About the role" paragraph reworded into the first person, so the candidate's stated goal is the employer's text
+- The resume's "Summary of Qualifications" walks through the JD's "What we are looking for" list in the JD's order, which is unlikely to happen by chance when someone writes from their own history
+- The resume gives its two earlier jobs one line each with unnamed employers, so there is no track record to compare the claims against</t>
         </is>
       </c>
       <c r="V3" t="inlineStr"/>
@@ -1129,8 +1131,8 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>- The nine duties listed in the posting appear as the nine bullets of the current job, in the same order and nearly the same words, which is what you get when a resume is written from the posting rather than from memory of the work
-- The employers are given only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no names, team sizes, numbers or incidents, so there is nothing here that could be checked
+          <t>- The resume's current-job bullets copy the JD's "What you will do" list: all nine duties, in the JD's order, in nearly the JD's words, which is what you get when a resume is written from the posting rather than from memory of the work
+- The resume names its employers only as "Leading Fintech Company" and "Global Technology Solutions Firm", with no team sizes, numbers or incidents, so there is nothing here that could be checked
 - Phone screen: ask about one specific Kubernetes upgrade they ran and what went wrong; someone who did the work will have a story</t>
         </is>
       </c>
@@ -1204,8 +1206,8 @@
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>- Each posting duty appears as a resume bullet with one word swapped ("Design, build and operate" becomes "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
-- Employers are given as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and there are no numbers anywhere, so nothing can be checked
+          <t>- The resume's current-job bullets restate the JD's "What you will do" list with one word swapped per bullet (the JD's "Design, build and operate" becomes the resume's "Architected and operated") in the same nine-bullet order, so the structure is the posting's even though the words differ
+- The resume names its employers as "Confidential Financial Services Company", "Enterprise Software Organization" and "Technology Consultancy", and gives no numbers anywhere, so nothing can be checked
 - Phone screen: ask which company it was and how much transaction volume it handled; a vague answer would confirm the concern</t>
         </is>
       </c>
@@ -1280,9 +1282,9 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>- The bullets follow the posting's order and wording with a percentage added to each, so the results look measured but the underlying claims are still the posting's
-- Every percentage is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
-- Employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
+          <t>- The resume's current-job bullets follow the JD's "What you will do" list in order and wording, with a percentage added to the end of each, so the results look measured but the underlying claims are still the posting's
+- Every percentage in the resume is a round number (80%, 60%, 50%, 40%, 90%, 100%, 300%) and every uptime figure is 99.99%, which is what invented metrics tend to look like
+- The resume's employers and dates look real, but no number is tied to a specific system, incident or time period, so the specifics may be decoration rather than evidence
 - Phone screen: pick two of the percentages and ask how they were measured; real ones come with a story, invented ones do not</t>
         </is>
       </c>
@@ -1415,9 +1417,9 @@
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>- Flagged only because most of the posting's acronyms appear, which is expected for someone who has this stack; the wording is the candidate's own and names tools the posting never mentions
-- The detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
-- Nothing suggests the wording came from the posting</t>
+          <t>- Flagged only because most of the JD's acronyms appear in the resume, which is expected for someone who has this stack; the resume's wording is its own and names tools the JD never mentions
+- The resume's detail is specific enough to check (14 AWS accounts, about $2B in payment volume, a 31% cost cut with the steps that got there), which is the opposite of what a resume written from a posting looks like
+- Nothing suggests the resume's wording came from the JD</t>
         </is>
       </c>
       <c r="V8" t="inlineStr"/>

</xml_diff>